<commit_message>
add drafted datastructure; renaming questions in survey
</commit_message>
<xml_diff>
--- a/surveys/biochar_survey_december_2025.xlsx
+++ b/surveys/biochar_survey_december_2025.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C4E07762-31C3-4608-9FAC-991CBC994265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4749A2D0-5141-4F66-B9AF-FE73F9785B49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="802">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2461" uniqueCount="801">
   <si>
     <t>type</t>
   </si>
@@ -1628,100 +1628,97 @@
     <t>C.4) During the seasons you applied biochar, how often did you apply it?</t>
   </si>
   <si>
+    <t>select_multiple yw1ml89</t>
+  </si>
+  <si>
+    <t>fertilizer_before_biochar</t>
+  </si>
+  <si>
+    <t>C.5) Prior to the season when you applied biochar, did you use fertilizer on that plot? (Select all that apply)</t>
+  </si>
+  <si>
+    <t>select_multiple pc1lg93</t>
+  </si>
+  <si>
+    <t>fertilizers_used_before_biocha</t>
+  </si>
+  <si>
+    <t>C.6) What kind of fertilizer did you use before biochar? (Select all that apply)</t>
+  </si>
+  <si>
+    <t>select_multiple td2jb01</t>
+  </si>
+  <si>
+    <t>fertilizers_used_with_biochar</t>
+  </si>
+  <si>
+    <t>C.7) When you applied biochar, did you also use another soil fertilizer in addition to biochar? (Select all that apply)</t>
+  </si>
+  <si>
+    <t>group_ad9ws92</t>
+  </si>
+  <si>
+    <t>Observation and Results</t>
+  </si>
+  <si>
+    <t>select_one sj05t62</t>
+  </si>
+  <si>
+    <t>biochar_used_on_different_area</t>
+  </si>
+  <si>
+    <t>D.1) On the crops where you used biochar, did you use it on some plots and not on other plots?</t>
+  </si>
+  <si>
+    <t>select_one xj9am89</t>
+  </si>
+  <si>
+    <t>noticed_difference</t>
+  </si>
+  <si>
+    <t>D.1.a) Did  you notice any difference between the plots where you used biochar and the plots where you did not or if you used biochar on only part of the plot did you see a difference in yield between where biochar was used and where it was not?</t>
+  </si>
+  <si>
+    <t>${biochar_used_on_different_area} = 'yes'</t>
+  </si>
+  <si>
+    <t>select_one hd83z15</t>
+  </si>
+  <si>
+    <t>significance_difference</t>
+  </si>
+  <si>
+    <t>D.1.b) How significant was the difference?</t>
+  </si>
+  <si>
+    <t>${noticed_difference} = 'yes' and ${biochar_used_on_different_area} = 'yes'</t>
+  </si>
+  <si>
+    <t>select_one hy91q54</t>
+  </si>
+  <si>
+    <t>noticeable_difference_in_yield</t>
+  </si>
+  <si>
+    <t>D.2) For crops for which you used biochar over the entire plot, can you judge whether there was a different in the yield from the crop was last cultivated, without biochar?</t>
+  </si>
+  <si>
+    <t>select_one ln0re11</t>
+  </si>
+  <si>
+    <t>significance_difference_yield</t>
+  </si>
+  <si>
+    <t>D.2.a) How significant was the difference in yield volume to the last yield without biochar?</t>
+  </si>
+  <si>
+    <t>${noticeable_difference_in_yield} = 'yes'</t>
+  </si>
+  <si>
     <t>most_affected_crop</t>
   </si>
   <si>
-    <t>C.5) If you used biochar on more than one crop, for which crops did it make the biggest difference? (Leave empty when cannot judge)</t>
-  </si>
-  <si>
-    <t>select_multiple yw1ml89</t>
-  </si>
-  <si>
-    <t>fertilizer_before_biochar</t>
-  </si>
-  <si>
-    <t>C.6) Before using biochar, did you use fertilizer? (Select all that apply)</t>
-  </si>
-  <si>
-    <t>select_multiple td2jb01</t>
-  </si>
-  <si>
-    <t>fertilizers_used_with_biochar</t>
-  </si>
-  <si>
-    <t>C.7) When you applied biochar, did you also use another soil fertilizer in addition to biochar? (Select all that apply)</t>
-  </si>
-  <si>
-    <t>select_multiple pc1lg93</t>
-  </si>
-  <si>
-    <t>fertilizers_used_before_biocha</t>
-  </si>
-  <si>
-    <t>C.8) What kind of fertilizer did you use before biochar? (Select all that apply)</t>
-  </si>
-  <si>
-    <t>group_ad9ws92</t>
-  </si>
-  <si>
-    <t>Observation and Results</t>
-  </si>
-  <si>
-    <t>select_one sj05t62</t>
-  </si>
-  <si>
-    <t>biochar_used_on_different_area</t>
-  </si>
-  <si>
-    <t>D.1) On the crops where you used biochar, did you use it on some plots and not one other plots?</t>
-  </si>
-  <si>
-    <t>select_one xj9am89</t>
-  </si>
-  <si>
-    <t>noticed_difference</t>
-  </si>
-  <si>
-    <t>D.2) Did  you notice any difference between the plots where you used biochar and the plots where you did not?</t>
-  </si>
-  <si>
-    <t>${biochar_used_on_different_area} = 'yes'</t>
-  </si>
-  <si>
-    <t>select_one hd83z15</t>
-  </si>
-  <si>
-    <t>significance_difference</t>
-  </si>
-  <si>
-    <t>D.2.a) How significant was the difference?</t>
-  </si>
-  <si>
-    <t>${noticed_difference} = 'yes'</t>
-  </si>
-  <si>
-    <t>select_one hy91q54</t>
-  </si>
-  <si>
-    <t>noticeable_difference_in_yield</t>
-  </si>
-  <si>
-    <t>D.3) For crops for which you used biochar over the entire plot, can you judge whether there was a different in the yield from the crop was last cultivated, without biochar?</t>
-  </si>
-  <si>
-    <t>select_one ln0re11</t>
-  </si>
-  <si>
-    <t>significance_difference_yield</t>
-  </si>
-  <si>
-    <t>D.3.a) How significant was the difference in yield volume to the last yield without biochar?</t>
-  </si>
-  <si>
-    <t>${noticeable_difference_in_yield} = 'yes'</t>
-  </si>
-  <si>
-    <t>D.4) If you used biochar on more than one crop, for which crops did it make the biggest difference? (Leave empty when cannot judge)</t>
+    <t>D.3) If you used biochar on more than one crop, for which crops did it make the biggest difference? (Leave empty when cannot judge)</t>
   </si>
   <si>
     <t>select_one po8ix91</t>
@@ -1730,13 +1727,13 @@
     <t>wants_to_continue_biochar</t>
   </si>
   <si>
-    <t>D.5) Do you plan to continue making and using biochar?</t>
+    <t>D.4) Do you plan to continue making and using biochar?</t>
   </si>
   <si>
     <t>reason_why_stopping_biochar</t>
   </si>
   <si>
-    <t>D.5.a) Why do you not plan to continue making biochar</t>
+    <t>D.4.a) Why do you not plan to continue making biochar</t>
   </si>
   <si>
     <t>${wants_to_continue_biochar} = 'no'</t>
@@ -1748,13 +1745,13 @@
     <t>simplification_for_biochar_use</t>
   </si>
   <si>
-    <t>D.6) What would make it easier for you to use biochar in future seasons?</t>
+    <t>D.5) What would make it easier for you to use biochar in future seasons?</t>
   </si>
   <si>
     <t>specified_simplifications</t>
   </si>
   <si>
-    <t>D.6.a) Please specify what would make it easier:</t>
+    <t>D.5.a) Please specify what would make it easier:</t>
   </si>
   <si>
     <t>selected(${simplification_for_biochar_use}, 'other')</t>
@@ -1766,7 +1763,7 @@
     <t>would_purchase_biochar</t>
   </si>
   <si>
-    <t>D.7) Would you purchase biochar if it were available?</t>
+    <t>D.6) Would you purchase biochar if it were available?</t>
   </si>
   <si>
     <t>select_multiple rm9rw73</t>
@@ -1775,7 +1772,7 @@
     <t>why_not_purchase_biochar</t>
   </si>
   <si>
-    <t>D.7.a) Why not?</t>
+    <t>D.6.a) Why not?</t>
   </si>
   <si>
     <t>${would_purchase_biochar} = 'no'</t>
@@ -1784,7 +1781,7 @@
     <t>specification_why_not_purchase</t>
   </si>
   <si>
-    <t>D.7.b) Please specify why not:</t>
+    <t>D.6.b) Please specify why not:</t>
   </si>
   <si>
     <t>selected(${why_not_purchase_biochar}, 'other')</t>
@@ -2787,7 +2784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F513"/>
+  <dimension ref="A1:F512"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.28515625" customWidth="1"/>
@@ -9766,13 +9763,13 @@
     </row>
     <row r="478" spans="1:6">
       <c r="A478" t="s">
-        <v>12</v>
+        <v>531</v>
       </c>
       <c r="B478" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="C478" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="D478" t="s">
         <v>11</v>
@@ -9783,13 +9780,13 @@
     </row>
     <row r="479" spans="1:6">
       <c r="A479" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B479" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="C479" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="D479" t="s">
         <v>11</v>
@@ -9800,13 +9797,13 @@
     </row>
     <row r="480" spans="1:6">
       <c r="A480" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B480" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="C480" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="D480" t="s">
         <v>11</v>
@@ -9817,131 +9814,128 @@
     </row>
     <row r="481" spans="1:5">
       <c r="A481" t="s">
-        <v>539</v>
-      </c>
-      <c r="B481" t="s">
-        <v>540</v>
-      </c>
-      <c r="C481" t="s">
-        <v>541</v>
-      </c>
-      <c r="D481" t="s">
-        <v>11</v>
-      </c>
-      <c r="E481" t="s">
-        <v>349</v>
+        <v>22</v>
       </c>
     </row>
     <row r="482" spans="1:5">
       <c r="A482" t="s">
-        <v>22</v>
+        <v>8</v>
+      </c>
+      <c r="B482" t="s">
+        <v>540</v>
+      </c>
+      <c r="C482" t="s">
+        <v>541</v>
+      </c>
+      <c r="D482" t="s">
+        <v>11</v>
+      </c>
+      <c r="E482" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="483" spans="1:5">
       <c r="A483" t="s">
-        <v>8</v>
+        <v>542</v>
       </c>
       <c r="B483" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C483" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="D483" t="s">
         <v>11</v>
-      </c>
-      <c r="E483" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="484" spans="1:5">
       <c r="A484" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B484" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="C484" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="D484" t="s">
         <v>11</v>
+      </c>
+      <c r="E484" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="485" spans="1:5">
       <c r="A485" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B485" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="C485" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="D485" t="s">
         <v>11</v>
       </c>
       <c r="E485" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="486" spans="1:5">
       <c r="A486" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B486" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="C486" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="D486" t="s">
         <v>11</v>
-      </c>
-      <c r="E486" t="s">
-        <v>554</v>
       </c>
     </row>
     <row r="487" spans="1:5">
       <c r="A487" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B487" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C487" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="D487" t="s">
         <v>11</v>
+      </c>
+      <c r="E487" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="488" spans="1:5">
       <c r="A488" t="s">
-        <v>558</v>
+        <v>12</v>
       </c>
       <c r="B488" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="C488" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="D488" t="s">
         <v>11</v>
-      </c>
-      <c r="E488" t="s">
-        <v>561</v>
       </c>
     </row>
     <row r="489" spans="1:5">
       <c r="A489" t="s">
-        <v>12</v>
+        <v>562</v>
       </c>
       <c r="B489" t="s">
-        <v>531</v>
+        <v>563</v>
       </c>
       <c r="C489" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="D489" t="s">
         <v>11</v>
@@ -9949,117 +9943,120 @@
     </row>
     <row r="490" spans="1:5">
       <c r="A490" t="s">
-        <v>563</v>
+        <v>12</v>
       </c>
       <c r="B490" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C490" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="D490" t="s">
         <v>11</v>
+      </c>
+      <c r="E490" t="s">
+        <v>567</v>
       </c>
     </row>
     <row r="491" spans="1:5">
       <c r="A491" t="s">
-        <v>12</v>
+        <v>568</v>
       </c>
       <c r="B491" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="C491" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="D491" t="s">
         <v>11</v>
-      </c>
-      <c r="E491" t="s">
-        <v>568</v>
       </c>
     </row>
     <row r="492" spans="1:5">
       <c r="A492" t="s">
-        <v>569</v>
+        <v>12</v>
       </c>
       <c r="B492" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C492" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="D492" t="s">
         <v>11</v>
+      </c>
+      <c r="E492" t="s">
+        <v>573</v>
       </c>
     </row>
     <row r="493" spans="1:5">
       <c r="A493" t="s">
-        <v>12</v>
+        <v>574</v>
       </c>
       <c r="B493" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="C493" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="D493" t="s">
         <v>11</v>
-      </c>
-      <c r="E493" t="s">
-        <v>574</v>
       </c>
     </row>
     <row r="494" spans="1:5">
       <c r="A494" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="B494" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="C494" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D494" t="s">
         <v>11</v>
+      </c>
+      <c r="E494" t="s">
+        <v>580</v>
       </c>
     </row>
     <row r="495" spans="1:5">
       <c r="A495" t="s">
-        <v>578</v>
+        <v>12</v>
       </c>
       <c r="B495" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="C495" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D495" t="s">
         <v>11</v>
       </c>
       <c r="E495" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="496" spans="1:5">
       <c r="A496" t="s">
-        <v>12</v>
-      </c>
-      <c r="B496" t="s">
-        <v>582</v>
-      </c>
-      <c r="C496" t="s">
-        <v>583</v>
-      </c>
-      <c r="D496" t="s">
-        <v>11</v>
-      </c>
-      <c r="E496" t="s">
-        <v>584</v>
+        <v>22</v>
       </c>
     </row>
     <row r="497" spans="1:5">
       <c r="A497" t="s">
-        <v>22</v>
+        <v>8</v>
+      </c>
+      <c r="B497" t="s">
+        <v>584</v>
+      </c>
+      <c r="C497" t="s">
+        <v>585</v>
+      </c>
+      <c r="D497" t="s">
+        <v>11</v>
+      </c>
+      <c r="E497" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="498" spans="1:5">
@@ -10067,38 +10064,35 @@
         <v>8</v>
       </c>
       <c r="B498" t="s">
-        <v>585</v>
-      </c>
-      <c r="C498" t="s">
         <v>586</v>
       </c>
       <c r="D498" t="s">
         <v>11</v>
-      </c>
-      <c r="E498" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="499" spans="1:5">
       <c r="A499" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="B499" t="s">
         <v>587</v>
       </c>
+      <c r="C499" t="s">
+        <v>588</v>
+      </c>
       <c r="D499" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="500" spans="1:5">
       <c r="A500" t="s">
-        <v>35</v>
+        <v>589</v>
       </c>
       <c r="B500" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="C500" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="D500" t="s">
         <v>11</v>
@@ -10106,13 +10100,13 @@
     </row>
     <row r="501" spans="1:5">
       <c r="A501" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B501" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C501" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="D501" t="s">
         <v>11</v>
@@ -10120,13 +10114,13 @@
     </row>
     <row r="502" spans="1:5">
       <c r="A502" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B502" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="C502" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="D502" t="s">
         <v>11</v>
@@ -10134,32 +10128,32 @@
     </row>
     <row r="503" spans="1:5">
       <c r="A503" t="s">
-        <v>590</v>
-      </c>
-      <c r="B503" t="s">
-        <v>595</v>
-      </c>
-      <c r="C503" t="s">
-        <v>596</v>
-      </c>
-      <c r="D503" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
     </row>
     <row r="504" spans="1:5">
       <c r="A504" t="s">
-        <v>22</v>
+        <v>35</v>
+      </c>
+      <c r="B504" t="s">
+        <v>596</v>
+      </c>
+      <c r="C504" t="s">
+        <v>521</v>
+      </c>
+      <c r="D504" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="505" spans="1:5">
       <c r="A505" t="s">
-        <v>35</v>
+        <v>597</v>
       </c>
       <c r="B505" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="C505" t="s">
-        <v>521</v>
+        <v>599</v>
       </c>
       <c r="D505" t="s">
         <v>11</v>
@@ -10167,32 +10161,32 @@
     </row>
     <row r="506" spans="1:5">
       <c r="A506" t="s">
-        <v>598</v>
-      </c>
-      <c r="B506" t="s">
-        <v>599</v>
-      </c>
-      <c r="C506" t="s">
-        <v>600</v>
-      </c>
-      <c r="D506" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
     </row>
     <row r="507" spans="1:5">
       <c r="A507" t="s">
-        <v>22</v>
+        <v>8</v>
+      </c>
+      <c r="B507" t="s">
+        <v>600</v>
+      </c>
+      <c r="C507" t="s">
+        <v>601</v>
+      </c>
+      <c r="D507" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="508" spans="1:5">
       <c r="A508" t="s">
-        <v>8</v>
+        <v>602</v>
       </c>
       <c r="B508" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="C508" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="D508" t="s">
         <v>11</v>
@@ -10200,68 +10194,54 @@
     </row>
     <row r="509" spans="1:5">
       <c r="A509" t="s">
-        <v>603</v>
+        <v>12</v>
       </c>
       <c r="B509" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="C509" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D509" t="s">
         <v>11</v>
+      </c>
+      <c r="E509" t="s">
+        <v>607</v>
       </c>
     </row>
     <row r="510" spans="1:5">
       <c r="A510" t="s">
-        <v>12</v>
+        <v>608</v>
       </c>
       <c r="B510" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="C510" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="D510" t="s">
         <v>11</v>
-      </c>
-      <c r="E510" t="s">
-        <v>608</v>
       </c>
     </row>
     <row r="511" spans="1:5">
       <c r="A511" t="s">
-        <v>609</v>
+        <v>12</v>
       </c>
       <c r="B511" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C511" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D511" t="s">
         <v>11</v>
+      </c>
+      <c r="E511" t="s">
+        <v>613</v>
       </c>
     </row>
     <row r="512" spans="1:5">
       <c r="A512" t="s">
-        <v>12</v>
-      </c>
-      <c r="B512" t="s">
-        <v>612</v>
-      </c>
-      <c r="C512" t="s">
-        <v>613</v>
-      </c>
-      <c r="D512" t="s">
-        <v>11</v>
-      </c>
-      <c r="E512" t="s">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="513" spans="1:1">
-      <c r="A513" t="s">
         <v>22</v>
       </c>
     </row>
@@ -10281,7 +10261,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -10290,1143 +10270,1143 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
+        <v>616</v>
+      </c>
+      <c r="B2" t="s">
         <v>617</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>618</v>
-      </c>
-      <c r="C2" t="s">
-        <v>619</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B3" t="s">
+        <v>619</v>
+      </c>
+      <c r="C3" t="s">
         <v>620</v>
-      </c>
-      <c r="C3" t="s">
-        <v>621</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
+        <v>621</v>
+      </c>
+      <c r="B4" t="s">
         <v>622</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>623</v>
-      </c>
-      <c r="C4" t="s">
-        <v>624</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B5" t="s">
+        <v>624</v>
+      </c>
+      <c r="C5" t="s">
         <v>625</v>
-      </c>
-      <c r="C5" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B6" t="s">
+        <v>626</v>
+      </c>
+      <c r="C6" t="s">
         <v>627</v>
-      </c>
-      <c r="C6" t="s">
-        <v>628</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B7" t="s">
+        <v>628</v>
+      </c>
+      <c r="C7" t="s">
         <v>629</v>
-      </c>
-      <c r="C7" t="s">
-        <v>630</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B8" t="s">
+        <v>630</v>
+      </c>
+      <c r="C8" t="s">
         <v>631</v>
-      </c>
-      <c r="C8" t="s">
-        <v>632</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B9" t="s">
+        <v>632</v>
+      </c>
+      <c r="C9" t="s">
         <v>633</v>
-      </c>
-      <c r="C9" t="s">
-        <v>634</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B10" t="s">
+        <v>634</v>
+      </c>
+      <c r="C10" t="s">
         <v>635</v>
-      </c>
-      <c r="C10" t="s">
-        <v>636</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
+        <v>636</v>
+      </c>
+      <c r="B11" t="s">
         <v>637</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>638</v>
-      </c>
-      <c r="C11" t="s">
-        <v>639</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B12" t="s">
+        <v>639</v>
+      </c>
+      <c r="C12" t="s">
         <v>640</v>
-      </c>
-      <c r="C12" t="s">
-        <v>641</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B13" t="s">
+        <v>641</v>
+      </c>
+      <c r="C13" t="s">
         <v>642</v>
-      </c>
-      <c r="C13" t="s">
-        <v>643</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B14" t="s">
+        <v>643</v>
+      </c>
+      <c r="C14" t="s">
         <v>644</v>
-      </c>
-      <c r="C14" t="s">
-        <v>645</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
+        <v>645</v>
+      </c>
+      <c r="B15" t="s">
         <v>646</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>647</v>
-      </c>
-      <c r="C15" t="s">
-        <v>648</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B16" t="s">
+        <v>648</v>
+      </c>
+      <c r="C16" t="s">
         <v>649</v>
-      </c>
-      <c r="C16" t="s">
-        <v>650</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B17" t="s">
+        <v>650</v>
+      </c>
+      <c r="C17" t="s">
         <v>651</v>
-      </c>
-      <c r="C17" t="s">
-        <v>652</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B18" t="s">
+        <v>652</v>
+      </c>
+      <c r="C18" t="s">
         <v>653</v>
-      </c>
-      <c r="C18" t="s">
-        <v>654</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B19" t="s">
+        <v>654</v>
+      </c>
+      <c r="C19" t="s">
         <v>655</v>
-      </c>
-      <c r="C19" t="s">
-        <v>656</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
+        <v>656</v>
+      </c>
+      <c r="B20" t="s">
         <v>657</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>658</v>
-      </c>
-      <c r="C20" t="s">
-        <v>659</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B21" t="s">
+        <v>659</v>
+      </c>
+      <c r="C21" t="s">
         <v>660</v>
-      </c>
-      <c r="C21" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B22" t="s">
+        <v>661</v>
+      </c>
+      <c r="C22" t="s">
         <v>662</v>
-      </c>
-      <c r="C22" t="s">
-        <v>663</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B23" t="s">
+        <v>663</v>
+      </c>
+      <c r="C23" t="s">
         <v>664</v>
-      </c>
-      <c r="C23" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B24" t="s">
+        <v>665</v>
+      </c>
+      <c r="C24" t="s">
         <v>666</v>
-      </c>
-      <c r="C24" t="s">
-        <v>667</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>667</v>
+      </c>
+      <c r="B25" t="s">
         <v>668</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>669</v>
-      </c>
-      <c r="C25" t="s">
-        <v>670</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B26" t="s">
+        <v>670</v>
+      </c>
+      <c r="C26" t="s">
         <v>671</v>
-      </c>
-      <c r="C26" t="s">
-        <v>672</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B27" t="s">
+        <v>672</v>
+      </c>
+      <c r="C27" t="s">
         <v>673</v>
-      </c>
-      <c r="C27" t="s">
-        <v>674</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
+        <v>674</v>
+      </c>
+      <c r="B28" t="s">
         <v>675</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>676</v>
-      </c>
-      <c r="C28" t="s">
-        <v>677</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B29" t="s">
+        <v>677</v>
+      </c>
+      <c r="C29" t="s">
         <v>678</v>
-      </c>
-      <c r="C29" t="s">
-        <v>679</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B30" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="C30" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
+        <v>680</v>
+      </c>
+      <c r="B31" t="s">
         <v>681</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>682</v>
-      </c>
-      <c r="C31" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B32" t="s">
+        <v>683</v>
+      </c>
+      <c r="C32" t="s">
         <v>684</v>
-      </c>
-      <c r="C32" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="B33" t="s">
+        <v>681</v>
+      </c>
+      <c r="C33" t="s">
         <v>682</v>
-      </c>
-      <c r="C33" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="B34" t="s">
+        <v>683</v>
+      </c>
+      <c r="C34" t="s">
         <v>684</v>
-      </c>
-      <c r="C34" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
+        <v>686</v>
+      </c>
+      <c r="B35" t="s">
         <v>687</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>688</v>
-      </c>
-      <c r="C35" t="s">
-        <v>689</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="B36" t="s">
+        <v>689</v>
+      </c>
+      <c r="C36" t="s">
         <v>690</v>
-      </c>
-      <c r="C36" t="s">
-        <v>691</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
+        <v>691</v>
+      </c>
+      <c r="B37" t="s">
         <v>692</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
         <v>693</v>
-      </c>
-      <c r="C37" t="s">
-        <v>694</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B38" t="s">
+        <v>694</v>
+      </c>
+      <c r="C38" t="s">
         <v>695</v>
-      </c>
-      <c r="C38" t="s">
-        <v>696</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
+        <v>696</v>
+      </c>
+      <c r="B39" t="s">
         <v>697</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>698</v>
-      </c>
-      <c r="C39" t="s">
-        <v>699</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="B40" t="s">
+        <v>699</v>
+      </c>
+      <c r="C40" t="s">
         <v>700</v>
-      </c>
-      <c r="C40" t="s">
-        <v>701</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="B41" t="s">
+        <v>701</v>
+      </c>
+      <c r="C41" t="s">
         <v>702</v>
-      </c>
-      <c r="C41" t="s">
-        <v>703</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
+        <v>703</v>
+      </c>
+      <c r="B42" t="s">
         <v>704</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>705</v>
-      </c>
-      <c r="C42" t="s">
-        <v>706</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B43" t="s">
+        <v>706</v>
+      </c>
+      <c r="C43" t="s">
         <v>707</v>
-      </c>
-      <c r="C43" t="s">
-        <v>708</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B44" t="s">
+        <v>708</v>
+      </c>
+      <c r="C44" t="s">
         <v>709</v>
-      </c>
-      <c r="C44" t="s">
-        <v>710</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
+        <v>710</v>
+      </c>
+      <c r="B45" t="s">
         <v>711</v>
       </c>
-      <c r="B45" t="s">
-        <v>712</v>
-      </c>
       <c r="C45" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
+        <v>710</v>
+      </c>
+      <c r="B46" t="s">
+        <v>712</v>
+      </c>
+      <c r="C46" t="s">
+        <v>712</v>
+      </c>
+      <c r="D46" t="s">
         <v>711</v>
-      </c>
-      <c r="B46" t="s">
-        <v>713</v>
-      </c>
-      <c r="C46" t="s">
-        <v>713</v>
-      </c>
-      <c r="D46" t="s">
-        <v>712</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="B47" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="C47" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="B48" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="C48" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
+        <v>715</v>
+      </c>
+      <c r="B49" t="s">
         <v>716</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C49" t="s">
         <v>717</v>
-      </c>
-      <c r="C49" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="B50" t="s">
+        <v>718</v>
+      </c>
+      <c r="C50" t="s">
         <v>719</v>
-      </c>
-      <c r="C50" t="s">
-        <v>720</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="B51" t="s">
+        <v>720</v>
+      </c>
+      <c r="C51" t="s">
         <v>721</v>
-      </c>
-      <c r="C51" t="s">
-        <v>722</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
+        <v>722</v>
+      </c>
+      <c r="B52" t="s">
         <v>723</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>724</v>
-      </c>
-      <c r="C52" t="s">
-        <v>725</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B53" t="s">
+        <v>725</v>
+      </c>
+      <c r="C53" t="s">
         <v>726</v>
-      </c>
-      <c r="C53" t="s">
-        <v>727</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B54" t="s">
+        <v>727</v>
+      </c>
+      <c r="C54" t="s">
         <v>728</v>
-      </c>
-      <c r="C54" t="s">
-        <v>729</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B55" t="s">
+        <v>725</v>
+      </c>
+      <c r="C55" t="s">
         <v>726</v>
-      </c>
-      <c r="C55" t="s">
-        <v>727</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B56" t="s">
+        <v>727</v>
+      </c>
+      <c r="C56" t="s">
         <v>728</v>
-      </c>
-      <c r="C56" t="s">
-        <v>729</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
+        <v>729</v>
+      </c>
+      <c r="B57" t="s">
         <v>730</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C57" t="s">
         <v>731</v>
-      </c>
-      <c r="C57" t="s">
-        <v>732</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="B58" t="s">
+        <v>681</v>
+      </c>
+      <c r="C58" t="s">
         <v>682</v>
-      </c>
-      <c r="C58" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="B59" t="s">
+        <v>683</v>
+      </c>
+      <c r="C59" t="s">
         <v>684</v>
-      </c>
-      <c r="C59" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="B60" t="s">
+        <v>681</v>
+      </c>
+      <c r="C60" t="s">
         <v>682</v>
-      </c>
-      <c r="C60" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="B61" t="s">
+        <v>683</v>
+      </c>
+      <c r="C61" t="s">
         <v>684</v>
-      </c>
-      <c r="C61" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
+        <v>734</v>
+      </c>
+      <c r="B62" t="s">
         <v>735</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C62" t="s">
         <v>736</v>
-      </c>
-      <c r="C62" t="s">
-        <v>737</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B63" t="s">
+        <v>737</v>
+      </c>
+      <c r="C63" t="s">
         <v>738</v>
-      </c>
-      <c r="C63" t="s">
-        <v>739</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B64" t="s">
+        <v>739</v>
+      </c>
+      <c r="C64" t="s">
         <v>740</v>
-      </c>
-      <c r="C64" t="s">
-        <v>741</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B65" t="s">
+        <v>741</v>
+      </c>
+      <c r="C65" t="s">
         <v>742</v>
-      </c>
-      <c r="C65" t="s">
-        <v>743</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="B66" t="s">
+        <v>681</v>
+      </c>
+      <c r="C66" t="s">
         <v>682</v>
-      </c>
-      <c r="C66" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="B67" t="s">
+        <v>683</v>
+      </c>
+      <c r="C67" t="s">
         <v>684</v>
-      </c>
-      <c r="C67" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B68" t="s">
+        <v>735</v>
+      </c>
+      <c r="C68" t="s">
         <v>736</v>
-      </c>
-      <c r="C68" t="s">
-        <v>737</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B69" t="s">
+        <v>737</v>
+      </c>
+      <c r="C69" t="s">
         <v>738</v>
-      </c>
-      <c r="C69" t="s">
-        <v>739</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B70" t="s">
+        <v>739</v>
+      </c>
+      <c r="C70" t="s">
         <v>740</v>
-      </c>
-      <c r="C70" t="s">
-        <v>741</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B71" t="s">
+        <v>741</v>
+      </c>
+      <c r="C71" t="s">
         <v>742</v>
-      </c>
-      <c r="C71" t="s">
-        <v>743</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B72" t="s">
+        <v>681</v>
+      </c>
+      <c r="C72" t="s">
         <v>682</v>
-      </c>
-      <c r="C72" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B73" t="s">
+        <v>683</v>
+      </c>
+      <c r="C73" t="s">
         <v>684</v>
-      </c>
-      <c r="C73" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
+        <v>745</v>
+      </c>
+      <c r="B74" t="s">
         <v>746</v>
       </c>
-      <c r="B74" t="s">
+      <c r="C74" t="s">
         <v>747</v>
-      </c>
-      <c r="C74" t="s">
-        <v>748</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
+        <v>748</v>
+      </c>
+      <c r="B75" t="s">
         <v>749</v>
       </c>
-      <c r="B75" t="s">
+      <c r="C75" t="s">
         <v>750</v>
-      </c>
-      <c r="C75" t="s">
-        <v>751</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B76" t="s">
+        <v>751</v>
+      </c>
+      <c r="C76" t="s">
         <v>752</v>
-      </c>
-      <c r="C76" t="s">
-        <v>753</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B77" t="s">
+        <v>753</v>
+      </c>
+      <c r="C77" t="s">
         <v>754</v>
-      </c>
-      <c r="C77" t="s">
-        <v>755</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B78" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="C78" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B79" t="s">
+        <v>681</v>
+      </c>
+      <c r="C79" t="s">
         <v>682</v>
-      </c>
-      <c r="C79" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B80" t="s">
+        <v>683</v>
+      </c>
+      <c r="C80" t="s">
         <v>684</v>
-      </c>
-      <c r="C80" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
+        <v>756</v>
+      </c>
+      <c r="B81" t="s">
         <v>757</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
         <v>758</v>
-      </c>
-      <c r="C81" t="s">
-        <v>759</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B82" t="s">
+        <v>759</v>
+      </c>
+      <c r="C82" t="s">
         <v>760</v>
-      </c>
-      <c r="C82" t="s">
-        <v>761</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B83" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="C83" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
+        <v>761</v>
+      </c>
+      <c r="B84" t="s">
         <v>762</v>
       </c>
-      <c r="B84" t="s">
+      <c r="C84" t="s">
         <v>763</v>
-      </c>
-      <c r="C84" t="s">
-        <v>764</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B85" t="s">
+        <v>764</v>
+      </c>
+      <c r="C85" t="s">
         <v>765</v>
-      </c>
-      <c r="C85" t="s">
-        <v>766</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B86" t="s">
+        <v>766</v>
+      </c>
+      <c r="C86" t="s">
         <v>767</v>
-      </c>
-      <c r="C86" t="s">
-        <v>768</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="B87" t="s">
+        <v>768</v>
+      </c>
+      <c r="C87" t="s">
         <v>769</v>
-      </c>
-      <c r="C87" t="s">
-        <v>770</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
+        <v>770</v>
+      </c>
+      <c r="B88" t="s">
         <v>771</v>
       </c>
-      <c r="B88" t="s">
+      <c r="C88" t="s">
         <v>772</v>
-      </c>
-      <c r="C88" t="s">
-        <v>773</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="B89" t="s">
+        <v>773</v>
+      </c>
+      <c r="C89" t="s">
         <v>774</v>
-      </c>
-      <c r="C89" t="s">
-        <v>775</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="B90" t="s">
+        <v>775</v>
+      </c>
+      <c r="C90" t="s">
         <v>776</v>
-      </c>
-      <c r="C90" t="s">
-        <v>777</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="B91" t="s">
+        <v>777</v>
+      </c>
+      <c r="C91" t="s">
         <v>778</v>
-      </c>
-      <c r="C91" t="s">
-        <v>779</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="B92" t="s">
+        <v>779</v>
+      </c>
+      <c r="C92" t="s">
         <v>780</v>
-      </c>
-      <c r="C92" t="s">
-        <v>781</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
+        <v>781</v>
+      </c>
+      <c r="B93" t="s">
         <v>782</v>
       </c>
-      <c r="B93" t="s">
+      <c r="C93" t="s">
         <v>783</v>
-      </c>
-      <c r="C93" t="s">
-        <v>784</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B94" t="s">
+        <v>784</v>
+      </c>
+      <c r="C94" t="s">
         <v>785</v>
-      </c>
-      <c r="C94" t="s">
-        <v>786</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B95" t="s">
+        <v>786</v>
+      </c>
+      <c r="C95" t="s">
         <v>787</v>
-      </c>
-      <c r="C95" t="s">
-        <v>788</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B96" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="C96" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" s="1" t="s">
+        <v>788</v>
+      </c>
+      <c r="B97" t="s">
         <v>789</v>
       </c>
-      <c r="B97" t="s">
+      <c r="C97" t="s">
         <v>790</v>
-      </c>
-      <c r="C97" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="B98" s="1" t="s">
+        <v>791</v>
+      </c>
+      <c r="C98" t="s">
         <v>792</v>
-      </c>
-      <c r="C98" t="s">
-        <v>793</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="B99" t="s">
+        <v>793</v>
+      </c>
+      <c r="C99" t="s">
         <v>794</v>
-      </c>
-      <c r="C99" t="s">
-        <v>795</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="B100" s="1" t="s">
+        <v>795</v>
+      </c>
+      <c r="C100" s="1" t="s">
         <v>796</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>797</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B101" t="s">
+        <v>681</v>
+      </c>
+      <c r="C101" t="s">
         <v>682</v>
-      </c>
-      <c r="C101" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B102" t="s">
+        <v>683</v>
+      </c>
+      <c r="C102" t="s">
         <v>684</v>
-      </c>
-      <c r="C102" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B103" t="s">
+        <v>681</v>
+      </c>
+      <c r="C103" t="s">
         <v>682</v>
-      </c>
-      <c r="C103" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="B104" t="s">
+        <v>683</v>
+      </c>
+      <c r="C104" t="s">
         <v>684</v>
-      </c>
-      <c r="C104" t="s">
-        <v>685</v>
       </c>
     </row>
   </sheetData>
@@ -11441,12 +11421,12 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add final dec 2025 survey
</commit_message>
<xml_diff>
--- a/surveys/biochar_survey_december_2025.xlsx
+++ b/surveys/biochar_survey_december_2025.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4749A2D0-5141-4F66-B9AF-FE73F9785B49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA1293E6-5814-446F-9EEC-C8993CFA9364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2461" uniqueCount="801">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2456" uniqueCount="798">
   <si>
     <t>type</t>
   </si>
@@ -1628,22 +1628,13 @@
     <t>C.4) During the seasons you applied biochar, how often did you apply it?</t>
   </si>
   <si>
-    <t>select_multiple yw1ml89</t>
-  </si>
-  <si>
-    <t>fertilizer_before_biochar</t>
-  </si>
-  <si>
-    <t>C.5) Prior to the season when you applied biochar, did you use fertilizer on that plot? (Select all that apply)</t>
-  </si>
-  <si>
     <t>select_multiple pc1lg93</t>
   </si>
   <si>
     <t>fertilizers_used_before_biocha</t>
   </si>
   <si>
-    <t>C.6) What kind of fertilizer did you use before biochar? (Select all that apply)</t>
+    <t>C.5) What kind of fertilizer did you use before biochar? (Select all that apply)</t>
   </si>
   <si>
     <t>select_multiple td2jb01</t>
@@ -1652,7 +1643,7 @@
     <t>fertilizers_used_with_biochar</t>
   </si>
   <si>
-    <t>C.7) When you applied biochar, did you also use another soil fertilizer in addition to biochar? (Select all that apply)</t>
+    <t>C.6) When you applied biochar, did you also use another soil fertilizer in addition to biochar? (Select all that apply)</t>
   </si>
   <si>
     <t>group_ad9ws92</t>
@@ -2784,7 +2775,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F512"/>
+  <dimension ref="A1:F511"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.28515625" customWidth="1"/>
@@ -9797,29 +9788,29 @@
     </row>
     <row r="480" spans="1:6">
       <c r="A480" t="s">
-        <v>537</v>
-      </c>
-      <c r="B480" t="s">
-        <v>538</v>
-      </c>
-      <c r="C480" t="s">
-        <v>539</v>
-      </c>
-      <c r="D480" t="s">
-        <v>11</v>
-      </c>
-      <c r="E480" t="s">
-        <v>349</v>
+        <v>22</v>
       </c>
     </row>
     <row r="481" spans="1:5">
       <c r="A481" t="s">
-        <v>22</v>
+        <v>8</v>
+      </c>
+      <c r="B481" t="s">
+        <v>537</v>
+      </c>
+      <c r="C481" t="s">
+        <v>538</v>
+      </c>
+      <c r="D481" t="s">
+        <v>11</v>
+      </c>
+      <c r="E481" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="482" spans="1:5">
       <c r="A482" t="s">
-        <v>8</v>
+        <v>539</v>
       </c>
       <c r="B482" t="s">
         <v>540</v>
@@ -9829,9 +9820,6 @@
       </c>
       <c r="D482" t="s">
         <v>11</v>
-      </c>
-      <c r="E482" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="483" spans="1:5">
@@ -9847,39 +9835,39 @@
       <c r="D483" t="s">
         <v>11</v>
       </c>
+      <c r="E483" t="s">
+        <v>545</v>
+      </c>
     </row>
     <row r="484" spans="1:5">
       <c r="A484" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B484" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="C484" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="D484" t="s">
         <v>11</v>
       </c>
       <c r="E484" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="485" spans="1:5">
       <c r="A485" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B485" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C485" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="D485" t="s">
         <v>11</v>
-      </c>
-      <c r="E485" t="s">
-        <v>552</v>
       </c>
     </row>
     <row r="486" spans="1:5">
@@ -9895,10 +9883,13 @@
       <c r="D486" t="s">
         <v>11</v>
       </c>
+      <c r="E486" t="s">
+        <v>556</v>
+      </c>
     </row>
     <row r="487" spans="1:5">
       <c r="A487" t="s">
-        <v>556</v>
+        <v>12</v>
       </c>
       <c r="B487" t="s">
         <v>557</v>
@@ -9909,13 +9900,10 @@
       <c r="D487" t="s">
         <v>11</v>
       </c>
-      <c r="E487" t="s">
-        <v>559</v>
-      </c>
     </row>
     <row r="488" spans="1:5">
       <c r="A488" t="s">
-        <v>12</v>
+        <v>559</v>
       </c>
       <c r="B488" t="s">
         <v>560</v>
@@ -9929,64 +9917,64 @@
     </row>
     <row r="489" spans="1:5">
       <c r="A489" t="s">
+        <v>12</v>
+      </c>
+      <c r="B489" t="s">
         <v>562</v>
       </c>
-      <c r="B489" t="s">
+      <c r="C489" t="s">
         <v>563</v>
       </c>
-      <c r="C489" t="s">
+      <c r="D489" t="s">
+        <v>11</v>
+      </c>
+      <c r="E489" t="s">
         <v>564</v>
-      </c>
-      <c r="D489" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="490" spans="1:5">
       <c r="A490" t="s">
-        <v>12</v>
+        <v>565</v>
       </c>
       <c r="B490" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C490" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="D490" t="s">
         <v>11</v>
-      </c>
-      <c r="E490" t="s">
-        <v>567</v>
       </c>
     </row>
     <row r="491" spans="1:5">
       <c r="A491" t="s">
+        <v>12</v>
+      </c>
+      <c r="B491" t="s">
         <v>568</v>
       </c>
-      <c r="B491" t="s">
+      <c r="C491" t="s">
         <v>569</v>
       </c>
-      <c r="C491" t="s">
+      <c r="D491" t="s">
+        <v>11</v>
+      </c>
+      <c r="E491" t="s">
         <v>570</v>
-      </c>
-      <c r="D491" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="492" spans="1:5">
       <c r="A492" t="s">
-        <v>12</v>
+        <v>571</v>
       </c>
       <c r="B492" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C492" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="D492" t="s">
         <v>11</v>
-      </c>
-      <c r="E492" t="s">
-        <v>573</v>
       </c>
     </row>
     <row r="493" spans="1:5">
@@ -10002,10 +9990,13 @@
       <c r="D493" t="s">
         <v>11</v>
       </c>
+      <c r="E493" t="s">
+        <v>577</v>
+      </c>
     </row>
     <row r="494" spans="1:5">
       <c r="A494" t="s">
-        <v>577</v>
+        <v>12</v>
       </c>
       <c r="B494" t="s">
         <v>578</v>
@@ -10022,24 +10013,24 @@
     </row>
     <row r="495" spans="1:5">
       <c r="A495" t="s">
-        <v>12</v>
-      </c>
-      <c r="B495" t="s">
-        <v>581</v>
-      </c>
-      <c r="C495" t="s">
-        <v>582</v>
-      </c>
-      <c r="D495" t="s">
-        <v>11</v>
-      </c>
-      <c r="E495" t="s">
-        <v>583</v>
+        <v>22</v>
       </c>
     </row>
     <row r="496" spans="1:5">
       <c r="A496" t="s">
-        <v>22</v>
+        <v>8</v>
+      </c>
+      <c r="B496" t="s">
+        <v>581</v>
+      </c>
+      <c r="C496" t="s">
+        <v>582</v>
+      </c>
+      <c r="D496" t="s">
+        <v>11</v>
+      </c>
+      <c r="E496" t="s">
+        <v>349</v>
       </c>
     </row>
     <row r="497" spans="1:5">
@@ -10047,24 +10038,21 @@
         <v>8</v>
       </c>
       <c r="B497" t="s">
-        <v>584</v>
-      </c>
-      <c r="C497" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="D497" t="s">
         <v>11</v>
-      </c>
-      <c r="E497" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="498" spans="1:5">
       <c r="A498" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="B498" t="s">
-        <v>586</v>
+        <v>584</v>
+      </c>
+      <c r="C498" t="s">
+        <v>585</v>
       </c>
       <c r="D498" t="s">
         <v>11</v>
@@ -10072,7 +10060,7 @@
     </row>
     <row r="499" spans="1:5">
       <c r="A499" t="s">
-        <v>35</v>
+        <v>586</v>
       </c>
       <c r="B499" t="s">
         <v>587</v>
@@ -10086,13 +10074,13 @@
     </row>
     <row r="500" spans="1:5">
       <c r="A500" t="s">
+        <v>586</v>
+      </c>
+      <c r="B500" t="s">
         <v>589</v>
       </c>
-      <c r="B500" t="s">
+      <c r="C500" t="s">
         <v>590</v>
-      </c>
-      <c r="C500" t="s">
-        <v>591</v>
       </c>
       <c r="D500" t="s">
         <v>11</v>
@@ -10100,13 +10088,13 @@
     </row>
     <row r="501" spans="1:5">
       <c r="A501" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="B501" t="s">
+        <v>591</v>
+      </c>
+      <c r="C501" t="s">
         <v>592</v>
-      </c>
-      <c r="C501" t="s">
-        <v>593</v>
       </c>
       <c r="D501" t="s">
         <v>11</v>
@@ -10114,32 +10102,32 @@
     </row>
     <row r="502" spans="1:5">
       <c r="A502" t="s">
-        <v>589</v>
-      </c>
-      <c r="B502" t="s">
-        <v>594</v>
-      </c>
-      <c r="C502" t="s">
-        <v>595</v>
-      </c>
-      <c r="D502" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
     </row>
     <row r="503" spans="1:5">
       <c r="A503" t="s">
-        <v>22</v>
+        <v>35</v>
+      </c>
+      <c r="B503" t="s">
+        <v>593</v>
+      </c>
+      <c r="C503" t="s">
+        <v>521</v>
+      </c>
+      <c r="D503" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="504" spans="1:5">
       <c r="A504" t="s">
-        <v>35</v>
+        <v>594</v>
       </c>
       <c r="B504" t="s">
+        <v>595</v>
+      </c>
+      <c r="C504" t="s">
         <v>596</v>
-      </c>
-      <c r="C504" t="s">
-        <v>521</v>
       </c>
       <c r="D504" t="s">
         <v>11</v>
@@ -10147,26 +10135,26 @@
     </row>
     <row r="505" spans="1:5">
       <c r="A505" t="s">
-        <v>597</v>
-      </c>
-      <c r="B505" t="s">
-        <v>598</v>
-      </c>
-      <c r="C505" t="s">
-        <v>599</v>
-      </c>
-      <c r="D505" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
     </row>
     <row r="506" spans="1:5">
       <c r="A506" t="s">
-        <v>22</v>
+        <v>8</v>
+      </c>
+      <c r="B506" t="s">
+        <v>597</v>
+      </c>
+      <c r="C506" t="s">
+        <v>598</v>
+      </c>
+      <c r="D506" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="507" spans="1:5">
       <c r="A507" t="s">
-        <v>8</v>
+        <v>599</v>
       </c>
       <c r="B507" t="s">
         <v>600</v>
@@ -10180,68 +10168,54 @@
     </row>
     <row r="508" spans="1:5">
       <c r="A508" t="s">
+        <v>12</v>
+      </c>
+      <c r="B508" t="s">
         <v>602</v>
       </c>
-      <c r="B508" t="s">
+      <c r="C508" t="s">
         <v>603</v>
       </c>
-      <c r="C508" t="s">
+      <c r="D508" t="s">
+        <v>11</v>
+      </c>
+      <c r="E508" t="s">
         <v>604</v>
-      </c>
-      <c r="D508" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="509" spans="1:5">
       <c r="A509" t="s">
-        <v>12</v>
+        <v>605</v>
       </c>
       <c r="B509" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="C509" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="D509" t="s">
         <v>11</v>
-      </c>
-      <c r="E509" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="510" spans="1:5">
       <c r="A510" t="s">
+        <v>12</v>
+      </c>
+      <c r="B510" t="s">
         <v>608</v>
       </c>
-      <c r="B510" t="s">
+      <c r="C510" t="s">
         <v>609</v>
       </c>
-      <c r="C510" t="s">
+      <c r="D510" t="s">
+        <v>11</v>
+      </c>
+      <c r="E510" t="s">
         <v>610</v>
-      </c>
-      <c r="D510" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="511" spans="1:5">
       <c r="A511" t="s">
-        <v>12</v>
-      </c>
-      <c r="B511" t="s">
-        <v>611</v>
-      </c>
-      <c r="C511" t="s">
-        <v>612</v>
-      </c>
-      <c r="D511" t="s">
-        <v>11</v>
-      </c>
-      <c r="E511" t="s">
-        <v>613</v>
-      </c>
-    </row>
-    <row r="512" spans="1:5">
-      <c r="A512" t="s">
         <v>22</v>
       </c>
     </row>
@@ -10261,7 +10235,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -10270,1143 +10244,1143 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="B2" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="C2" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
+        <v>613</v>
+      </c>
+      <c r="B3" t="s">
         <v>616</v>
       </c>
-      <c r="B3" t="s">
-        <v>619</v>
-      </c>
       <c r="C3" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="B4" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="C4" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
+        <v>618</v>
+      </c>
+      <c r="B5" t="s">
         <v>621</v>
       </c>
-      <c r="B5" t="s">
-        <v>624</v>
-      </c>
       <c r="C5" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="B6" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="C6" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="B7" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="C7" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="B8" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="C8" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="B9" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="C9" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="B10" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="C10" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="B11" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="C11" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
+        <v>633</v>
+      </c>
+      <c r="B12" t="s">
         <v>636</v>
       </c>
-      <c r="B12" t="s">
-        <v>639</v>
-      </c>
       <c r="C12" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="B13" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="C13" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="B14" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="C14" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="B15" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="C15" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
+        <v>642</v>
+      </c>
+      <c r="B16" t="s">
         <v>645</v>
       </c>
-      <c r="B16" t="s">
-        <v>648</v>
-      </c>
       <c r="C16" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="B17" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="C17" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="B18" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="C18" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="B19" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="C19" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="B20" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="C20" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
+        <v>653</v>
+      </c>
+      <c r="B21" t="s">
         <v>656</v>
       </c>
-      <c r="B21" t="s">
-        <v>659</v>
-      </c>
       <c r="C21" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="B22" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="C22" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="B23" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="C23" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="B24" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C24" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="B25" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="C25" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
+        <v>664</v>
+      </c>
+      <c r="B26" t="s">
         <v>667</v>
       </c>
-      <c r="B26" t="s">
-        <v>670</v>
-      </c>
       <c r="C26" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="B27" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="C27" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="B28" t="s">
-        <v>675</v>
+        <v>672</v>
       </c>
       <c r="C28" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
+        <v>671</v>
+      </c>
+      <c r="B29" t="s">
         <v>674</v>
       </c>
-      <c r="B29" t="s">
-        <v>677</v>
-      </c>
       <c r="C29" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="B30" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="C30" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
       <c r="B31" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="C31" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
+        <v>677</v>
+      </c>
+      <c r="B32" t="s">
         <v>680</v>
       </c>
-      <c r="B32" t="s">
-        <v>683</v>
-      </c>
       <c r="C32" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="B33" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="C33" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="B34" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="C34" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="B35" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="C35" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
+        <v>683</v>
+      </c>
+      <c r="B36" t="s">
         <v>686</v>
       </c>
-      <c r="B36" t="s">
-        <v>689</v>
-      </c>
       <c r="C36" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
       <c r="B37" t="s">
-        <v>692</v>
+        <v>689</v>
       </c>
       <c r="C37" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
+        <v>688</v>
+      </c>
+      <c r="B38" t="s">
         <v>691</v>
       </c>
-      <c r="B38" t="s">
-        <v>694</v>
-      </c>
       <c r="C38" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="B39" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="C39" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
+        <v>693</v>
+      </c>
+      <c r="B40" t="s">
         <v>696</v>
       </c>
-      <c r="B40" t="s">
-        <v>699</v>
-      </c>
       <c r="C40" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="B41" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="C41" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="B42" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="C42" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
+        <v>700</v>
+      </c>
+      <c r="B43" t="s">
         <v>703</v>
       </c>
-      <c r="B43" t="s">
-        <v>706</v>
-      </c>
       <c r="C43" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="B44" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="C44" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="B45" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="C45" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="B46" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="C46" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="D46" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
+        <v>707</v>
+      </c>
+      <c r="B47" t="s">
         <v>710</v>
       </c>
-      <c r="B47" t="s">
-        <v>713</v>
-      </c>
       <c r="C47" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="B48" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="C48" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="B49" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="C49" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
+        <v>712</v>
+      </c>
+      <c r="B50" t="s">
         <v>715</v>
       </c>
-      <c r="B50" t="s">
-        <v>718</v>
-      </c>
       <c r="C50" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="B51" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="C51" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="B52" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="C52" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
+        <v>719</v>
+      </c>
+      <c r="B53" t="s">
         <v>722</v>
       </c>
-      <c r="B53" t="s">
-        <v>725</v>
-      </c>
       <c r="C53" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="B54" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="C54" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="B55" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="C55" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="B56" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="C56" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="B57" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="C57" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="B58" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="C58" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="B59" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="C59" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="B60" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="C60" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="B61" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="C61" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="B62" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="C62" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
+        <v>731</v>
+      </c>
+      <c r="B63" t="s">
         <v>734</v>
       </c>
-      <c r="B63" t="s">
-        <v>737</v>
-      </c>
       <c r="C63" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="B64" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="C64" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="B65" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="C65" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="B66" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="C66" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="B67" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="C67" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="B68" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="C68" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="B69" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="C69" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="B70" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
       <c r="C70" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="B71" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="C71" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="B72" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="C72" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="B73" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="C73" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="B74" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="C74" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="B75" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="C75" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
+        <v>745</v>
+      </c>
+      <c r="B76" t="s">
         <v>748</v>
       </c>
-      <c r="B76" t="s">
-        <v>751</v>
-      </c>
       <c r="C76" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="B77" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="C77" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="B78" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="C78" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B79" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="C79" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="B80" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="C80" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="B81" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="C81" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
+        <v>753</v>
+      </c>
+      <c r="B82" t="s">
         <v>756</v>
       </c>
-      <c r="B82" t="s">
-        <v>759</v>
-      </c>
       <c r="C82" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="B83" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="C83" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="B84" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="C84" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
+        <v>758</v>
+      </c>
+      <c r="B85" t="s">
         <v>761</v>
       </c>
-      <c r="B85" t="s">
-        <v>764</v>
-      </c>
       <c r="C85" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="B86" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="C86" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="B87" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="C87" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="B88" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="C88" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
+        <v>767</v>
+      </c>
+      <c r="B89" t="s">
         <v>770</v>
       </c>
-      <c r="B89" t="s">
-        <v>773</v>
-      </c>
       <c r="C89" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="B90" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
       <c r="C90" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="B91" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="C91" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="B92" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="C92" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="B93" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="C93" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
+        <v>778</v>
+      </c>
+      <c r="B94" t="s">
         <v>781</v>
       </c>
-      <c r="B94" t="s">
-        <v>784</v>
-      </c>
       <c r="C94" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="B95" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="C95" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="B96" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="C96" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" s="1" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="B97" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C97" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="B98" s="1" t="s">
         <v>788</v>
       </c>
-      <c r="B98" s="1" t="s">
-        <v>791</v>
-      </c>
       <c r="C98" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" s="1" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="B99" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="C99" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" s="1" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="B101" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="C101" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="B102" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="C102" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="B103" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="C103" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="B104" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="C104" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
     </row>
   </sheetData>
@@ -11421,12 +11395,12 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
     </row>
   </sheetData>

</xml_diff>